<commit_message>
Modified table template to include highlighting of blanks
</commit_message>
<xml_diff>
--- a/To Add v2/1Table_Template.xlsx
+++ b/To Add v2/1Table_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\To Add v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C4A77A-D448-438D-8257-50BDAFE1CEEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82DA5618-9EC6-4BC0-ACBE-576AFD0E1674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="7725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -160,7 +160,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -437,15 +445,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:T7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.08984375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -453,7 +461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -505,7 +513,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:20" x14ac:dyDescent="0.35">
       <c r="S3" t="s">
         <v>4</v>
       </c>
@@ -514,7 +522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>5</v>
       </c>
@@ -556,7 +564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:20" x14ac:dyDescent="0.35">
       <c r="S5" t="s">
         <v>7</v>
       </c>
@@ -565,7 +573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>8</v>
       </c>
@@ -606,7 +614,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>21</v>
       </c>
@@ -658,6 +666,11 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C7:L147">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(C7))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>